<commit_message>
Plantilla: agregar columna Proveedor (7 cols)
</commit_message>
<xml_diff>
--- a/public/Pazque_plantilla_productos.xlsx
+++ b/public/Pazque_plantilla_productos.xlsx
@@ -98,12 +98,24 @@
         </r>
       </text>
     </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Proveedor o marca del producto. Opcional, podés dejarlo vacío.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t xml:space="preserve">Nombre</t>
   </si>
@@ -123,6 +135,9 @@
     <t xml:space="preserve">Unidad</t>
   </si>
   <si>
+    <t xml:space="preserve">Proveedor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Queso Colonia x 4kg</t>
   </si>
   <si>
@@ -135,6 +150,9 @@
     <t xml:space="preserve">unidad</t>
   </si>
   <si>
+    <t xml:space="preserve">Lácteos del Sur</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jamón cocido x 1kg</t>
   </si>
   <si>
@@ -147,6 +165,9 @@
     <t xml:space="preserve">kg</t>
   </si>
   <si>
+    <t xml:space="preserve">Frigorífico Centro</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aceite girasol 900ml</t>
   </si>
   <si>
@@ -156,6 +177,9 @@
     <t xml:space="preserve">Almacén</t>
   </si>
   <si>
+    <t xml:space="preserve">Distribuidora Norte</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cómo completar esta plantilla</t>
   </si>
   <si>
@@ -190,6 +214,12 @@
   </si>
   <si>
     <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El 'Proveedor' es opcional: podés dejarlo vacío si no lo usás.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
   </si>
   <si>
     <t xml:space="preserve">Guardá el archivo y subilo en Pazque desde la pantalla Importar.</t>
@@ -632,7 +662,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -641,6 +671,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -662,16 +693,19 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>580</v>
@@ -680,18 +714,21 @@
         <v>24</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>410</v>
@@ -700,18 +737,21 @@
         <v>60</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>95</v>
@@ -720,7 +760,10 @@
         <v>120</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -730,6 +773,7 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
@@ -738,6 +782,7 @@
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
@@ -746,6 +791,7 @@
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6"/>
@@ -754,6 +800,7 @@
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
@@ -762,6 +809,7 @@
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
@@ -770,6 +818,7 @@
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
@@ -778,6 +827,7 @@
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
@@ -786,6 +836,7 @@
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -804,7 +855,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -813,61 +864,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B1" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="10" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plantilla: bordes guia hasta fila 50
</commit_message>
<xml_diff>
--- a/public/Pazque_plantilla_productos.xlsx
+++ b/public/Pazque_plantilla_productos.xlsx
@@ -115,7 +115,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t xml:space="preserve">Nombre</t>
   </si>
@@ -220,6 +220,12 @@
   </si>
   <si>
     <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si necesitás más filas, seguí escribiendo hacia abajo: no hay límite, el sistema las lee todas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
   </si>
   <si>
     <t xml:space="preserve">Guardá el archivo y subilo en Pazque desde la pantalla Importar.</t>
@@ -662,7 +668,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -837,6 +843,348 @@
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6"/>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6"/>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6"/>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="6"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -855,7 +1203,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -924,9 +1272,17 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10" t="s">
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>36</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="10" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>